<commit_message>
Concentra as visitas sorteadas em 03/10 e sincroniza o projeto com o registro prévio
Emenda 4 do registro prévio: as duas unidades da São Jogue são visitadas
no sábado, 03/10, com hora de início sorteada, duração fixa de 3 horas e
no mínimo 2 horas entre os inícios; retorno no domingo, 18/10. Script e
planilha do sorteio refeitos (mesma semente), metodologia e cronogramas
atualizados.

Projeto de pesquisa: H5 passa a comparar com a cesta do próprio
estabelecimento e a validação da codificação segue o registro prévio
(segunda pessoa ou recodificação após 14 dias); quadro de itens ganha as
notas por aspecto, horário de funcionamento e localização em shopping.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_data/processed/[D] Contagem direta de ocupacao/contagem_sorteio_visitas.xlsx
+++ b/_data/processed/[D] Contagem direta de ocupacao/contagem_sorteio_visitas.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Instruções" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Parâmetros" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Dias e horas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Horas" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Retorno" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Sorteio" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Registro" sheetId="6" state="visible" r:id="rId6"/>
@@ -103,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -135,12 +135,12 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -148,6 +148,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -527,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -560,7 +566,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2. Nas abas Dias e horas e Retorno, marque "não" nas colunas amarelas de cada unidade para os dias e horas em que ela não abre. Faça isso ANTES de abrir a aba Sorteio: mudar a lista depois de ver o resultado invalida o sorteio.</t>
+          <t>2. Na aba Horas, marque "não" nas colunas amarelas de cada unidade para as horas de início em que ela não fica aberta pelas 3 horas seguintes. Na aba Retorno, marque "não" para os dias em que ela não abre. Faça isso ANTES de abrir a aba Sorteio: mudar a lista depois de ver o resultado invalida o sorteio.</t>
         </is>
       </c>
     </row>
@@ -598,67 +604,74 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>• Visitas sorteadas entre 02/10 e 04/10/2026. Cada combinação de dia e hora de início (12h00 a 19h00, de hora em hora) é uma possibilidade. As duas unidades ficam em dias diferentes.</t>
+          <t>• Visitas sorteadas no sábado, 03/10/2026, as duas unidades no mesmo dia. Só a hora de início é sorteada (12h00 a 19h00, de hora em hora).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>• Um número sorteado define qual unidade escolhe primeiro. Cada unidade fica com a combinação aberta de menor número aleatório; a segunda unidade não pode ficar no mesmo dia da primeira.</t>
+          <t>• Duração fixa de 3 horas. As horas de início das duas unidades distam no mínimo 2 horas.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>• Visita de retorno: 15 dias depois da sorteada, na mesma unidade e na mesma hora de início (17/10 a 19/10/2026). Se a unidade estiver fechada, a visita passa ao dia seguinte de funcionamento.</t>
+          <t>• Um número sorteado define qual unidade escolhe primeiro. A primeira fica com a hora aberta de menor número aleatório; a segunda, com a hora aberta de menor número aleatório que respeite a distância mínima.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>• Em cada visita, registrar o número da NFC-e no início e no fim, e o horário de início e de fim. A diferença entre os números da visita sorteada e da de retorno dá as notas emitidas no intervalo.</t>
+          <t>• Visita de retorno: 15 dias depois, no domingo, 18/10/2026, na mesma unidade e na mesma hora de início. Se a unidade estiver fechada, a visita passa ao dia seguinte de funcionamento.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>• Visitas sem duração fixa, do lado de fora do estabelecimento, com contagem a cada 30 minutos.</t>
+          <t>• Em cada visita, registrar o número da NFC-e no início e no fim, e o horário de início e de fim. A diferença entre os números da visita sorteada e da de retorno dá as notas emitidas no intervalo.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>• Visitas do lado de fora do estabelecimento, com contagem a cada 30 minutos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>• Os números aleatórios foram gerados com semente fixa (20260916) pelo script _src/[D] Contagem direta de ocupacao/build_contagem_sorteio.py e não devem ser editados.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Legenda de cores</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Fundo amarelo: célula para preencher. Texto azul: valor fixo (dado ou número sorteado). Texto preto: fórmula. Texto verde: fórmula que busca dado de outra aba.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Fonte das datas de pagamento: Governo da Bahia, Tabela de Pagamentos 2026 dos servidores estaduais (servidores.rhbahia.ba.gov.br/tabela-de-pagamentos-2026), consultada em 17/09/2026. Setembro: ativos 30/09, inativos e pensionistas 29/09. Outubro: ativos 30/10, inativos e pensionistas 29/10.</t>
         </is>
@@ -675,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -744,30 +757,30 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Primeiro dia das visitas sorteadas</t>
+          <t>Dia das visitas sorteadas</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Sexta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Último dia das visitas sorteadas</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="n">
-        <v>46299</v>
+          <t>Duração de cada visita (horas)</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Fixa</t>
         </is>
       </c>
     </row>
@@ -813,6 +826,21 @@
       <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Contados a partir da visita sorteada</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Distância mínima entre as horas de início (horas)</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Entre as duas unidades</t>
         </is>
       </c>
     </row>
@@ -827,21 +855,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Combinações de dia e hora de início das visitas sorteadas</t>
+          <t>Horas de início possíveis das visitas sorteadas (03/10/2026)</t>
         </is>
       </c>
     </row>
@@ -853,27 +880,22 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Hora</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Dia da semana</t>
+          <t>Hora de início</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Hora de início</t>
+          <t>Unidade 1 aberta por 3 h?</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Unidade 1 aberta?</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>Unidade 2 aberta?</t>
+          <t>Unidade 2 aberta por 3 h?</t>
         </is>
       </c>
     </row>
@@ -881,24 +903,20 @@
       <c r="A3" s="10" t="n">
         <v>0.6825255929118569</v>
       </c>
-      <c r="B3" s="8" t="n">
-        <v>46297</v>
-      </c>
-      <c r="C3" s="11">
-        <f>CHOOSE(WEEKDAY(B3,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="B3" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>12h00</t>
         </is>
       </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
@@ -908,24 +926,20 @@
       <c r="A4" s="10" t="n">
         <v>0.9420456376610188</v>
       </c>
-      <c r="B4" s="8" t="n">
-        <v>46297</v>
-      </c>
-      <c r="C4" s="11">
-        <f>CHOOSE(WEEKDAY(B4,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="B4" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>13h00</t>
         </is>
       </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
@@ -935,24 +949,20 @@
       <c r="A5" s="10" t="n">
         <v>0.8701514202626593</v>
       </c>
-      <c r="B5" s="8" t="n">
-        <v>46297</v>
-      </c>
-      <c r="C5" s="11">
-        <f>CHOOSE(WEEKDAY(B5,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="B5" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>14h00</t>
         </is>
       </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
@@ -962,24 +972,20 @@
       <c r="A6" s="10" t="n">
         <v>0.1085408879036384</v>
       </c>
-      <c r="B6" s="8" t="n">
-        <v>46297</v>
-      </c>
-      <c r="C6" s="11">
-        <f>CHOOSE(WEEKDAY(B6,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="B6" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>15h00</t>
         </is>
       </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
@@ -989,24 +995,20 @@
       <c r="A7" s="10" t="n">
         <v>0.5044517982097884</v>
       </c>
-      <c r="B7" s="8" t="n">
-        <v>46297</v>
-      </c>
-      <c r="C7" s="11">
-        <f>CHOOSE(WEEKDAY(B7,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="B7" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>16h00</t>
         </is>
       </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
@@ -1016,24 +1018,20 @@
       <c r="A8" s="10" t="n">
         <v>0.8663027492310936</v>
       </c>
-      <c r="B8" s="8" t="n">
-        <v>46297</v>
-      </c>
-      <c r="C8" s="11">
-        <f>CHOOSE(WEEKDAY(B8,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="B8" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>17h00</t>
         </is>
       </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
@@ -1043,24 +1041,20 @@
       <c r="A9" s="10" t="n">
         <v>0.5899372207964796</v>
       </c>
-      <c r="B9" s="8" t="n">
-        <v>46297</v>
-      </c>
-      <c r="C9" s="11">
-        <f>CHOOSE(WEEKDAY(B9,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="B9" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>18h00</t>
         </is>
       </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
@@ -1070,456 +1064,20 @@
       <c r="A10" s="10" t="n">
         <v>0.6618768317480069</v>
       </c>
-      <c r="B10" s="8" t="n">
-        <v>46297</v>
-      </c>
-      <c r="C10" s="11">
-        <f>CHOOSE(WEEKDAY(B10,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="B10" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>19h00</t>
         </is>
       </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="n">
-        <v>0.6030938513646101</v>
-      </c>
-      <c r="B11" s="8" t="n">
-        <v>46298</v>
-      </c>
-      <c r="C11" s="11">
-        <f>CHOOSE(WEEKDAY(B11,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>12h00</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="n">
-        <v>0.7351310965538348</v>
-      </c>
-      <c r="B12" s="8" t="n">
-        <v>46298</v>
-      </c>
-      <c r="C12" s="11">
-        <f>CHOOSE(WEEKDAY(B12,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>13h00</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="n">
-        <v>0.6125826800980299</v>
-      </c>
-      <c r="B13" s="8" t="n">
-        <v>46298</v>
-      </c>
-      <c r="C13" s="11">
-        <f>CHOOSE(WEEKDAY(B13,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>14h00</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="n">
-        <v>0.2430836278838648</v>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>46298</v>
-      </c>
-      <c r="C14" s="11">
-        <f>CHOOSE(WEEKDAY(B14,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>15h00</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="n">
-        <v>0.1730766924901449</v>
-      </c>
-      <c r="B15" s="8" t="n">
-        <v>46298</v>
-      </c>
-      <c r="C15" s="11">
-        <f>CHOOSE(WEEKDAY(B15,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>16h00</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="n">
-        <v>0.2688377912382225</v>
-      </c>
-      <c r="B16" s="8" t="n">
-        <v>46298</v>
-      </c>
-      <c r="C16" s="11">
-        <f>CHOOSE(WEEKDAY(B16,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>17h00</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="n">
-        <v>0.6384763378898026</v>
-      </c>
-      <c r="B17" s="8" t="n">
-        <v>46298</v>
-      </c>
-      <c r="C17" s="11">
-        <f>CHOOSE(WEEKDAY(B17,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>18h00</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="n">
-        <v>0.7979611189056641</v>
-      </c>
-      <c r="B18" s="8" t="n">
-        <v>46298</v>
-      </c>
-      <c r="C18" s="11">
-        <f>CHOOSE(WEEKDAY(B18,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>19h00</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="n">
-        <v>0.6368536235161361</v>
-      </c>
-      <c r="B19" s="8" t="n">
-        <v>46299</v>
-      </c>
-      <c r="C19" s="11">
-        <f>CHOOSE(WEEKDAY(B19,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>12h00</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="n">
-        <v>0.5305828736421826</v>
-      </c>
-      <c r="B20" s="8" t="n">
-        <v>46299</v>
-      </c>
-      <c r="C20" s="11">
-        <f>CHOOSE(WEEKDAY(B20,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>13h00</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="n">
-        <v>0.405083223577504</v>
-      </c>
-      <c r="B21" s="8" t="n">
-        <v>46299</v>
-      </c>
-      <c r="C21" s="11">
-        <f>CHOOSE(WEEKDAY(B21,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>14h00</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="n">
-        <v>0.1278970371792419</v>
-      </c>
-      <c r="B22" s="8" t="n">
-        <v>46299</v>
-      </c>
-      <c r="C22" s="11">
-        <f>CHOOSE(WEEKDAY(B22,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>15h00</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="10" t="n">
-        <v>0.4845666963325101</v>
-      </c>
-      <c r="B23" s="8" t="n">
-        <v>46299</v>
-      </c>
-      <c r="C23" s="11">
-        <f>CHOOSE(WEEKDAY(B23,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>16h00</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="n">
-        <v>0.805315083187461</v>
-      </c>
-      <c r="B24" s="8" t="n">
-        <v>46299</v>
-      </c>
-      <c r="C24" s="11">
-        <f>CHOOSE(WEEKDAY(B24,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>17h00</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="n">
-        <v>0.1822396280224478</v>
-      </c>
-      <c r="B25" s="8" t="n">
-        <v>46299</v>
-      </c>
-      <c r="C25" s="11">
-        <f>CHOOSE(WEEKDAY(B25,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D25" s="12" t="inlineStr">
-        <is>
-          <t>18h00</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="n">
-        <v>0.4764214824658619</v>
-      </c>
-      <c r="B26" s="8" t="n">
-        <v>46299</v>
-      </c>
-      <c r="C26" s="11">
-        <f>CHOOSE(WEEKDAY(B26,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t>19h00</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
@@ -1527,7 +1085,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E3:F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D3:E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"sim,não"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1541,7 +1099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1581,9 +1139,9 @@
     </row>
     <row r="3">
       <c r="A3" s="8" t="n">
-        <v>46312</v>
-      </c>
-      <c r="B3" s="11">
+        <v>46313</v>
+      </c>
+      <c r="B3" s="12">
         <f>CHOOSE(WEEKDAY(A3,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
         <v/>
       </c>
@@ -1600,9 +1158,9 @@
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
-        <v>46313</v>
-      </c>
-      <c r="B4" s="11">
+        <v>46314</v>
+      </c>
+      <c r="B4" s="12">
         <f>CHOOSE(WEEKDAY(A4,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
         <v/>
       </c>
@@ -1619,9 +1177,9 @@
     </row>
     <row r="5">
       <c r="A5" s="8" t="n">
-        <v>46314</v>
-      </c>
-      <c r="B5" s="11">
+        <v>46315</v>
+      </c>
+      <c r="B5" s="12">
         <f>CHOOSE(WEEKDAY(A5,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
         <v/>
       </c>
@@ -1631,82 +1189,6 @@
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="n">
-        <v>46315</v>
-      </c>
-      <c r="B6" s="11">
-        <f>CHOOSE(WEEKDAY(A6,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="n">
-        <v>46316</v>
-      </c>
-      <c r="B7" s="11">
-        <f>CHOOSE(WEEKDAY(A7,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="n">
-        <v>46317</v>
-      </c>
-      <c r="B8" s="11">
-        <f>CHOOSE(WEEKDAY(A8,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="B9" s="11">
-        <f>CHOOSE(WEEKDAY(A9,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo")</f>
-        <v/>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
@@ -1714,7 +1196,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C3:D9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C3:D5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"sim,não"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1728,7 +1210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1738,6 +1220,7 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1783,12 +1266,17 @@
           <t>Número aleatório</t>
         </is>
       </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="n">
+      <c r="A3" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Sorteada</t>
         </is>
@@ -1798,27 +1286,31 @@
         <v/>
       </c>
       <c r="D3" s="14">
-        <f>IFERROR(INDEX('Dias e horas'!$B$3:$B$26,MATCH(G3,'Dias e horas'!$A$3:$A$26,0)),"sem combinação")</f>
-        <v/>
-      </c>
-      <c r="E3" s="11">
+        <f>Parâmetros!$B$6</f>
+        <v/>
+      </c>
+      <c r="E3" s="12">
         <f>IFERROR(CHOOSE(WEEKDAY(D3,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo"),"")</f>
         <v/>
       </c>
       <c r="F3" s="13">
-        <f>IFERROR(INDEX('Dias e horas'!$D$3:$D$26,MATCH(G3,'Dias e horas'!$A$3:$A$26,0)),"")</f>
+        <f>IFERROR(INDEX(Horas!$C$3:$C$10,MATCH(G3,Horas!$A$3:$A$10,0)),"sem hora válida")</f>
         <v/>
       </c>
       <c r="G3" s="15">
-        <f>IF(C3=Parâmetros!$B$4,_xlfn.MINIFS('Dias e horas'!$A$3:$A$26,'Dias e horas'!$E$3:$E$26,"sim"),_xlfn.MINIFS('Dias e horas'!$A$3:$A$26,'Dias e horas'!$F$3:$F$26,"sim"))</f>
+        <f>IF(C3=Parâmetros!$B$4,_xlfn.MINIFS(Horas!$A$3:$A$10,Horas!$D$3:$D$10,"sim"),_xlfn.MINIFS(Horas!$A$3:$A$10,Horas!$E$3:$E$10,"sim"))</f>
+        <v/>
+      </c>
+      <c r="H3" s="16">
+        <f>IFERROR(INDEX(Horas!$B$3:$B$10,MATCH(G3,Horas!$A$3:$A$10,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n">
+      <c r="A4" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Sorteada</t>
         </is>
@@ -1828,102 +1320,114 @@
         <v/>
       </c>
       <c r="D4" s="14">
-        <f>IFERROR(INDEX('Dias e horas'!$B$3:$B$26,MATCH(G4,'Dias e horas'!$A$3:$A$26,0)),"sem combinação")</f>
-        <v/>
-      </c>
-      <c r="E4" s="11">
+        <f>Parâmetros!$B$6</f>
+        <v/>
+      </c>
+      <c r="E4" s="12">
         <f>IFERROR(CHOOSE(WEEKDAY(D4,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo"),"")</f>
         <v/>
       </c>
       <c r="F4" s="13">
-        <f>IFERROR(INDEX('Dias e horas'!$D$3:$D$26,MATCH(G4,'Dias e horas'!$A$3:$A$26,0)),"")</f>
+        <f>IFERROR(INDEX(Horas!$C$3:$C$10,MATCH(G4,Horas!$A$3:$A$10,0)),"sem hora válida")</f>
         <v/>
       </c>
       <c r="G4" s="15">
-        <f>IF(C4=Parâmetros!$B$4,_xlfn.MINIFS('Dias e horas'!$A$3:$A$26,'Dias e horas'!$E$3:$E$26,"sim",'Dias e horas'!$B$3:$B$26,"&lt;&gt;"&amp;D3),_xlfn.MINIFS('Dias e horas'!$A$3:$A$26,'Dias e horas'!$F$3:$F$26,"sim",'Dias e horas'!$B$3:$B$26,"&lt;&gt;"&amp;D3))</f>
+        <f>MIN(IF(_xlfn.MINIFS(Horas!$A$3:$A$10,IF(C4=Parâmetros!$B$4,Horas!$D$3:$D$10,Horas!$E$3:$E$10),"sim",Horas!$B$3:$B$10,"&lt;="&amp;(H3-Parâmetros!$B$11))=0,9,_xlfn.MINIFS(Horas!$A$3:$A$10,IF(C4=Parâmetros!$B$4,Horas!$D$3:$D$10,Horas!$E$3:$E$10),"sim",Horas!$B$3:$B$10,"&lt;="&amp;(H3-Parâmetros!$B$11))),IF(_xlfn.MINIFS(Horas!$A$3:$A$10,IF(C4=Parâmetros!$B$4,Horas!$D$3:$D$10,Horas!$E$3:$E$10),"sim",Horas!$B$3:$B$10,"&gt;="&amp;(H3+Parâmetros!$B$11))=0,9,_xlfn.MINIFS(Horas!$A$3:$A$10,IF(C4=Parâmetros!$B$4,Horas!$D$3:$D$10,Horas!$E$3:$E$10),"sim",Horas!$B$3:$B$10,"&gt;="&amp;(H3+Parâmetros!$B$11))))</f>
+        <v/>
+      </c>
+      <c r="H4" s="16">
+        <f>IFERROR(INDEX(Horas!$B$3:$B$10,MATCH(G4,Horas!$A$3:$A$10,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Retorno da visita 1</t>
         </is>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="12">
         <f>C3</f>
         <v/>
       </c>
       <c r="D5" s="14">
-        <f>IFERROR(INDEX(Retorno!$A$3:$A$9,MATCH(1,INDEX((Retorno!$A$3:$A$9&gt;=(D3+Parâmetros!$B$10))*((C5=Parâmetros!$B$4)*(Retorno!$C$3:$C$9="sim")+(C5&lt;&gt;Parâmetros!$B$4)*(Retorno!$D$3:$D$9="sim")),0),0)),"sem dia de retorno")</f>
-        <v/>
-      </c>
-      <c r="E5" s="11">
+        <f>IFERROR(INDEX(Retorno!$A$3:$A$5,MATCH(1,INDEX((Retorno!$A$3:$A$5&gt;=(D3+Parâmetros!$B$10))*((C5=Parâmetros!$B$4)*(Retorno!$C$3:$C$5="sim")+(C5&lt;&gt;Parâmetros!$B$4)*(Retorno!$D$3:$D$5="sim")),0),0)),"sem dia de retorno")</f>
+        <v/>
+      </c>
+      <c r="E5" s="12">
         <f>IFERROR(CHOOSE(WEEKDAY(D5,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo"),"")</f>
         <v/>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="12">
         <f>F3</f>
         <v/>
       </c>
       <c r="G5" s="6" t="n"/>
+      <c r="H5" s="17">
+        <f>H3</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Retorno da visita 2</t>
         </is>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="12">
         <f>C4</f>
         <v/>
       </c>
       <c r="D6" s="14">
-        <f>IFERROR(INDEX(Retorno!$A$3:$A$9,MATCH(1,INDEX((Retorno!$A$3:$A$9&gt;=(D4+Parâmetros!$B$10))*((C6=Parâmetros!$B$4)*(Retorno!$C$3:$C$9="sim")+(C6&lt;&gt;Parâmetros!$B$4)*(Retorno!$D$3:$D$9="sim")),0),0)),"sem dia de retorno")</f>
-        <v/>
-      </c>
-      <c r="E6" s="11">
+        <f>IFERROR(INDEX(Retorno!$A$3:$A$5,MATCH(1,INDEX((Retorno!$A$3:$A$5&gt;=(D4+Parâmetros!$B$10))*((C6=Parâmetros!$B$4)*(Retorno!$C$3:$C$5="sim")+(C6&lt;&gt;Parâmetros!$B$4)*(Retorno!$D$3:$D$5="sim")),0),0)),"sem dia de retorno")</f>
+        <v/>
+      </c>
+      <c r="E6" s="12">
         <f>IFERROR(CHOOSE(WEEKDAY(D6,2),"segunda","terça","quarta","quinta","sexta","sábado","domingo"),"")</f>
         <v/>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="12">
         <f>F4</f>
         <v/>
       </c>
       <c r="G6" s="6" t="n"/>
+      <c r="H6" s="17">
+        <f>H4</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Conferência</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Visitas por unidade (deve dar 2 e 2):</t>
         </is>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="19">
         <f>Parâmetros!$B$4&amp;": "&amp;COUNTIF($C$3:$C$6,Parâmetros!$B$4)&amp;" | "&amp;Parâmetros!$B$5&amp;": "&amp;COUNTIF($C$3:$C$6,Parâmetros!$B$5)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>Visitas sorteadas em dias diferentes:</t>
-        </is>
-      </c>
-      <c r="D10" s="17">
-        <f>IF(AND(ISNUMBER(D3),ISNUMBER(D4),D3&lt;&gt;D4),"sim","não")</f>
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>Horas de início com a distância mínima:</t>
+        </is>
+      </c>
+      <c r="D10" s="19">
+        <f>IF(AND(ISNUMBER(H3),ISNUMBER(H4)),IF(ABS(H3-H4)&gt;=Parâmetros!$B$11,"sim","não"),"não")</f>
         <v/>
       </c>
     </row>
@@ -1963,12 +1467,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Data do sorteio:</t>
         </is>
       </c>
-      <c r="B2" s="18" t="n"/>
+      <c r="B2" s="20" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -2033,60 +1537,60 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="n"/>
-      <c r="B5" s="19" t="n"/>
-      <c r="C5" s="19" t="n"/>
-      <c r="D5" s="19" t="n"/>
-      <c r="E5" s="19" t="n"/>
-      <c r="F5" s="19" t="n"/>
-      <c r="G5" s="19" t="n"/>
-      <c r="H5" s="19" t="n"/>
-      <c r="I5" s="19" t="n"/>
-      <c r="J5" s="19" t="n"/>
-      <c r="K5" s="19" t="n"/>
-      <c r="L5" s="19" t="n"/>
+      <c r="A5" s="21" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="21" t="n"/>
+      <c r="H5" s="21" t="n"/>
+      <c r="I5" s="21" t="n"/>
+      <c r="J5" s="21" t="n"/>
+      <c r="K5" s="21" t="n"/>
+      <c r="L5" s="21" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n"/>
-      <c r="B6" s="19" t="n"/>
-      <c r="C6" s="19" t="n"/>
-      <c r="D6" s="19" t="n"/>
-      <c r="E6" s="19" t="n"/>
-      <c r="F6" s="19" t="n"/>
-      <c r="G6" s="19" t="n"/>
-      <c r="H6" s="19" t="n"/>
-      <c r="I6" s="19" t="n"/>
-      <c r="J6" s="19" t="n"/>
-      <c r="K6" s="19" t="n"/>
-      <c r="L6" s="19" t="n"/>
+      <c r="A6" s="21" t="n"/>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="21" t="n"/>
+      <c r="G6" s="21" t="n"/>
+      <c r="H6" s="21" t="n"/>
+      <c r="I6" s="21" t="n"/>
+      <c r="J6" s="21" t="n"/>
+      <c r="K6" s="21" t="n"/>
+      <c r="L6" s="21" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n"/>
-      <c r="B7" s="19" t="n"/>
-      <c r="C7" s="19" t="n"/>
-      <c r="D7" s="19" t="n"/>
-      <c r="E7" s="19" t="n"/>
-      <c r="F7" s="19" t="n"/>
-      <c r="G7" s="19" t="n"/>
-      <c r="H7" s="19" t="n"/>
-      <c r="I7" s="19" t="n"/>
-      <c r="J7" s="19" t="n"/>
-      <c r="K7" s="19" t="n"/>
-      <c r="L7" s="19" t="n"/>
+      <c r="A7" s="21" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="21" t="n"/>
+      <c r="G7" s="21" t="n"/>
+      <c r="H7" s="21" t="n"/>
+      <c r="I7" s="21" t="n"/>
+      <c r="J7" s="21" t="n"/>
+      <c r="K7" s="21" t="n"/>
+      <c r="L7" s="21" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="19" t="n"/>
-      <c r="C8" s="19" t="n"/>
-      <c r="D8" s="19" t="n"/>
-      <c r="E8" s="19" t="n"/>
-      <c r="F8" s="19" t="n"/>
-      <c r="G8" s="19" t="n"/>
-      <c r="H8" s="19" t="n"/>
-      <c r="I8" s="19" t="n"/>
-      <c r="J8" s="19" t="n"/>
-      <c r="K8" s="19" t="n"/>
-      <c r="L8" s="19" t="n"/>
+      <c r="A8" s="21" t="n"/>
+      <c r="B8" s="21" t="n"/>
+      <c r="C8" s="21" t="n"/>
+      <c r="D8" s="21" t="n"/>
+      <c r="E8" s="21" t="n"/>
+      <c r="F8" s="21" t="n"/>
+      <c r="G8" s="21" t="n"/>
+      <c r="H8" s="21" t="n"/>
+      <c r="I8" s="21" t="n"/>
+      <c r="J8" s="21" t="n"/>
+      <c r="K8" s="21" t="n"/>
+      <c r="L8" s="21" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>